<commit_message>
Phase 3: compare all arms and add robustness outputs
</commit_message>
<xml_diff>
--- a/outputs/tables/ame_bootstrap_results_approach.xlsx
+++ b/outputs/tables/ame_bootstrap_results_approach.xlsx
@@ -458,25 +458,25 @@
         <v>0.00251190834760991</v>
       </c>
       <c r="D2" t="n">
-        <v>0.00079104652948844</v>
+        <v>0.000930818546608357</v>
       </c>
       <c r="E2" t="n">
-        <v>3.1754242689546</v>
+        <v>2.69860152310308</v>
       </c>
       <c r="F2" t="n">
-        <v>0.00149617569428796</v>
+        <v>0.00696314956670199</v>
       </c>
       <c r="G2" t="n">
-        <v>0.00218102769810028</v>
+        <v>0.00117193200690993</v>
       </c>
       <c r="H2" t="n">
-        <v>0.00391130061834026</v>
+        <v>0.00434472632118441</v>
       </c>
       <c r="I2" t="n">
         <v>0.95</v>
       </c>
       <c r="J2" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="K2" t="n">
         <v>0</v>
@@ -493,25 +493,25 @@
         <v>-0.00069196025705529</v>
       </c>
       <c r="D3" t="n">
-        <v>0.000833504328214822</v>
+        <v>0.000847327512496271</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.830181960227265</v>
+        <v>-0.816638486122963</v>
       </c>
       <c r="F3" t="n">
-        <v>0.406435913120611</v>
+        <v>0.414135054427015</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.00122988427724751</v>
+        <v>-0.00228738694827236</v>
       </c>
       <c r="H3" t="n">
-        <v>0.000649172131958622</v>
+        <v>0.000785702906272928</v>
       </c>
       <c r="I3" t="n">
         <v>0.95</v>
       </c>
       <c r="J3" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
@@ -528,25 +528,25 @@
         <v>0.00435631214436828</v>
       </c>
       <c r="D4" t="n">
-        <v>0.000426372470403002</v>
+        <v>0.00093675563584539</v>
       </c>
       <c r="E4" t="n">
-        <v>10.2171515441669</v>
+        <v>4.65042533791308</v>
       </c>
       <c r="F4" t="n">
-        <v>0.00000000000000000000000166151530538022</v>
+        <v>0.00000331251151053464</v>
       </c>
       <c r="G4" t="n">
-        <v>0.00355402993933631</v>
+        <v>0.00301926341014717</v>
       </c>
       <c r="H4" t="n">
-        <v>0.00457483026118233</v>
+        <v>0.00629108585641372</v>
       </c>
       <c r="I4" t="n">
         <v>0.95</v>
       </c>
       <c r="J4" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
@@ -563,25 +563,25 @@
         <v>-0.00687929233689501</v>
       </c>
       <c r="D5" t="n">
-        <v>0.000828341853852998</v>
+        <v>0.00113375793944294</v>
       </c>
       <c r="E5" t="n">
-        <v>-8.30489526141444</v>
+        <v>-6.06769055154322</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0000000000000000999075388216742</v>
+        <v>0.00000000129762617606165</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.00738580363017081</v>
+        <v>-0.00942668914397172</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.00553738874196547</v>
+        <v>-0.00522816402303002</v>
       </c>
       <c r="I5" t="n">
         <v>0.95</v>
       </c>
       <c r="J5" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="K5" t="n">
         <v>0</v>
@@ -598,25 +598,25 @@
         <v>-0.0108227154955342</v>
       </c>
       <c r="D6" t="n">
-        <v>0.0013073942420378</v>
+        <v>0.00128220374353288</v>
       </c>
       <c r="E6" t="n">
-        <v>-8.27808104666661</v>
+        <v>-8.44071431714445</v>
       </c>
       <c r="F6" t="n">
-        <v>0.000000000000000125176025553048</v>
+        <v>0.0000000000000000315404169737342</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.0126322526548258</v>
+        <v>-0.0142928004860602</v>
       </c>
       <c r="H6" t="n">
-        <v>-0.00957750978898896</v>
+        <v>-0.00914851218727705</v>
       </c>
       <c r="I6" t="n">
         <v>0.95</v>
       </c>
       <c r="J6" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="K6" t="n">
         <v>0</v>
@@ -633,25 +633,25 @@
         <v>0.0085177938226603</v>
       </c>
       <c r="D7" t="n">
-        <v>0.000964676841613421</v>
+        <v>0.00108005693487494</v>
       </c>
       <c r="E7" t="n">
-        <v>8.82968622778826</v>
+        <v>7.88643037938237</v>
       </c>
       <c r="F7" t="n">
-        <v>0.00000000000000000104969776281726</v>
+        <v>0.00000000000000310952902121557</v>
       </c>
       <c r="G7" t="n">
-        <v>0.00666129082837849</v>
+        <v>0.00698620359472585</v>
       </c>
       <c r="H7" t="n">
-        <v>0.00911661446816121</v>
+        <v>0.0112255591113743</v>
       </c>
       <c r="I7" t="n">
         <v>0.95</v>
       </c>
       <c r="J7" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="K7" t="n">
         <v>0</v>
@@ -668,25 +668,25 @@
         <v>0.0038707284099903</v>
       </c>
       <c r="D8" t="n">
-        <v>0.00172129672462792</v>
+        <v>0.00188325338450077</v>
       </c>
       <c r="E8" t="n">
-        <v>2.24872815628404</v>
+        <v>2.05534127369503</v>
       </c>
       <c r="F8" t="n">
-        <v>0.0245297966706829</v>
+        <v>0.0398460534267934</v>
       </c>
       <c r="G8" t="n">
-        <v>0.00180195628244933</v>
+        <v>0.000324601691883314</v>
       </c>
       <c r="H8" t="n">
-        <v>0.00614903518365768</v>
+        <v>0.0074001699375416</v>
       </c>
       <c r="I8" t="n">
         <v>0.95</v>
       </c>
       <c r="J8" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="K8" t="n">
         <v>0</v>
@@ -703,25 +703,25 @@
         <v>-0.00238285906883262</v>
       </c>
       <c r="D9" t="n">
-        <v>0.00178547108158793</v>
+        <v>0.0016739394421119</v>
       </c>
       <c r="E9" t="n">
-        <v>-1.33458284113647</v>
+        <v>-1.42350374743923</v>
       </c>
       <c r="F9" t="n">
-        <v>0.182012917051153</v>
+        <v>0.154590176546692</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.00538285098141283</v>
+        <v>-0.00593989962039739</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.00114564073212228</v>
+        <v>0.000382412918374141</v>
       </c>
       <c r="I9" t="n">
         <v>0.95</v>
       </c>
       <c r="J9" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="K9" t="n">
         <v>0</v>
@@ -738,25 +738,25 @@
         <v>0.00798420219459716</v>
       </c>
       <c r="D10" t="n">
-        <v>0.00181008044980238</v>
+        <v>0.0019894205029175</v>
       </c>
       <c r="E10" t="n">
-        <v>4.41096537751616</v>
+        <v>4.01333060702263</v>
       </c>
       <c r="F10" t="n">
-        <v>0.0000102910773813826</v>
+        <v>0.0000598679696155497</v>
       </c>
       <c r="G10" t="n">
-        <v>0.00690983546598008</v>
+        <v>0.0044904221445647</v>
       </c>
       <c r="H10" t="n">
-        <v>0.0112799234930763</v>
+        <v>0.0116820761784076</v>
       </c>
       <c r="I10" t="n">
         <v>0.95</v>
       </c>
       <c r="J10" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="K10" t="n">
         <v>0</v>
@@ -773,25 +773,25 @@
         <v>-0.0137567233580021</v>
       </c>
       <c r="D11" t="n">
-        <v>0.00196792275130722</v>
+        <v>0.00166328693298608</v>
       </c>
       <c r="E11" t="n">
-        <v>-6.99047935131801</v>
+        <v>-8.27080588753549</v>
       </c>
       <c r="F11" t="n">
-        <v>0.00000000000273948615698679</v>
+        <v>0.000000000000000133056531943828</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.0156448479258248</v>
+        <v>-0.0168029725589851</v>
       </c>
       <c r="H11" t="n">
-        <v>-0.0111248078878855</v>
+        <v>-0.0112141470180955</v>
       </c>
       <c r="I11" t="n">
         <v>0.95</v>
       </c>
       <c r="J11" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="K11" t="n">
         <v>0</v>
@@ -808,25 +808,25 @@
         <v>-0.0172845085344577</v>
       </c>
       <c r="D12" t="n">
-        <v>0.00152581389938471</v>
+        <v>0.00211534327623754</v>
       </c>
       <c r="E12" t="n">
-        <v>-11.3280581212608</v>
+        <v>-8.1710182591266</v>
       </c>
       <c r="F12" t="n">
-        <v>0.00000000000000000000000000000952940168981976</v>
+        <v>0.000000000000000305797345228089</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.019553182648406</v>
+        <v>-0.0226360004657024</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.0161247315928786</v>
+        <v>-0.013899291859683</v>
       </c>
       <c r="I12" t="n">
         <v>0.95</v>
       </c>
       <c r="J12" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="K12" t="n">
         <v>0</v>
@@ -843,25 +843,25 @@
         <v>0.0104491832013978</v>
       </c>
       <c r="D13" t="n">
-        <v>0.00170889143545993</v>
+        <v>0.00177859133979313</v>
       </c>
       <c r="E13" t="n">
-        <v>6.11459744286533</v>
+        <v>5.87497699309224</v>
       </c>
       <c r="F13" t="n">
-        <v>0.000000000968010067278484</v>
+        <v>0.00000000422902077801826</v>
       </c>
       <c r="G13" t="n">
-        <v>0.00870567617369414</v>
+        <v>0.00772738925867471</v>
       </c>
       <c r="H13" t="n">
-        <v>0.0127164418189806</v>
+        <v>0.0140579836882148</v>
       </c>
       <c r="I13" t="n">
         <v>0.95</v>
       </c>
       <c r="J13" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="K13" t="n">
         <v>0</v>
@@ -878,25 +878,25 @@
         <v>0.00231682921083476</v>
       </c>
       <c r="D14" t="n">
-        <v>0.00339116348121207</v>
+        <v>0.00335604259936959</v>
       </c>
       <c r="E14" t="n">
-        <v>0.683195966125078</v>
+        <v>0.690345590747258</v>
       </c>
       <c r="F14" t="n">
-        <v>0.494483021282758</v>
+        <v>0.489976883920176</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.00228008119867054</v>
+        <v>-0.00218148936409277</v>
       </c>
       <c r="H14" t="n">
-        <v>0.00548360003691341</v>
+        <v>0.0106377787935817</v>
       </c>
       <c r="I14" t="n">
         <v>0.95</v>
       </c>
       <c r="J14" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="K14" t="n">
         <v>0</v>
@@ -913,25 +913,25 @@
         <v>0.00210399998609066</v>
       </c>
       <c r="D15" t="n">
-        <v>0.00135090154785743</v>
+        <v>0.00261371489200546</v>
       </c>
       <c r="E15" t="n">
-        <v>1.55747840353552</v>
+        <v>0.804984504058243</v>
       </c>
       <c r="F15" t="n">
-        <v>0.119356944152966</v>
+        <v>0.420828621977363</v>
       </c>
       <c r="G15" t="n">
-        <v>-0.0022189656386194</v>
+        <v>-0.00313030750068823</v>
       </c>
       <c r="H15" t="n">
-        <v>0.00119720150383866</v>
+        <v>0.0071964725250886</v>
       </c>
       <c r="I15" t="n">
         <v>0.95</v>
       </c>
       <c r="J15" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="K15" t="n">
         <v>0</v>
@@ -948,25 +948,25 @@
         <v>0.00986257482305979</v>
       </c>
       <c r="D16" t="n">
-        <v>0.00131176379213299</v>
+        <v>0.00360094032742184</v>
       </c>
       <c r="E16" t="n">
-        <v>7.51856003512854</v>
+        <v>2.73888871413792</v>
       </c>
       <c r="F16" t="n">
-        <v>0.0000000000000553828136764464</v>
+        <v>0.00616472366626185</v>
       </c>
       <c r="G16" t="n">
-        <v>0.00917570311366249</v>
+        <v>0.00329599673490454</v>
       </c>
       <c r="H16" t="n">
-        <v>0.012394451457349</v>
+        <v>0.0177941261837955</v>
       </c>
       <c r="I16" t="n">
         <v>0.95</v>
       </c>
       <c r="J16" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="K16" t="n">
         <v>0</v>
@@ -983,25 +983,25 @@
         <v>-0.0288497543851824</v>
       </c>
       <c r="D17" t="n">
-        <v>0.00316955822491761</v>
+        <v>0.00361768907789319</v>
       </c>
       <c r="E17" t="n">
-        <v>-9.10213737623713</v>
+        <v>-7.9746362288225</v>
       </c>
       <c r="F17" t="n">
-        <v>0.0000000000000000000885713097162689</v>
+        <v>0.00000000000000152830288501597</v>
       </c>
       <c r="G17" t="n">
-        <v>-0.030140839302717</v>
+        <v>-0.0361844554022485</v>
       </c>
       <c r="H17" t="n">
-        <v>-0.0223216478397497</v>
+        <v>-0.0214722063302412</v>
       </c>
       <c r="I17" t="n">
         <v>0.95</v>
       </c>
       <c r="J17" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="K17" t="n">
         <v>0</v>
@@ -1018,25 +1018,25 @@
         <v>-0.0349315983597081</v>
       </c>
       <c r="D18" t="n">
-        <v>0.00337252798291415</v>
+        <v>0.00374766762942674</v>
       </c>
       <c r="E18" t="n">
-        <v>-10.3576897024066</v>
+        <v>-9.32089016790728</v>
       </c>
       <c r="F18" t="n">
-        <v>0.00000000000000000000000038617689861546</v>
+        <v>0.0000000000000000000115368268259306</v>
       </c>
       <c r="G18" t="n">
-        <v>-0.0348968933338954</v>
+        <v>-0.0427657022813374</v>
       </c>
       <c r="H18" t="n">
-        <v>-0.0281734724620527</v>
+        <v>-0.0282205219749131</v>
       </c>
       <c r="I18" t="n">
         <v>0.95</v>
       </c>
       <c r="J18" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="K18" t="n">
         <v>0</v>
@@ -1053,25 +1053,25 @@
         <v>0.0242044128199862</v>
       </c>
       <c r="D19" t="n">
-        <v>0.00381034615427362</v>
+        <v>0.00233757908056197</v>
       </c>
       <c r="E19" t="n">
-        <v>6.35228712563003</v>
+        <v>10.3544787088732</v>
       </c>
       <c r="F19" t="n">
-        <v>0.000000000212136881436971</v>
+        <v>0.000000000000000000000000399356059847022</v>
       </c>
       <c r="G19" t="n">
-        <v>0.0182864097426901</v>
+        <v>0.0197805134661398</v>
       </c>
       <c r="H19" t="n">
-        <v>0.0274289024266138</v>
+        <v>0.0288846731980314</v>
       </c>
       <c r="I19" t="n">
         <v>0.95</v>
       </c>
       <c r="J19" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="K19" t="n">
         <v>0</v>
@@ -1088,25 +1088,25 @@
         <v>0.00906109734923069</v>
       </c>
       <c r="D20" t="n">
-        <v>0.00421762639140361</v>
+        <v>0.00544938783008424</v>
       </c>
       <c r="E20" t="n">
-        <v>2.14838786282708</v>
+        <v>1.66277344020321</v>
       </c>
       <c r="F20" t="n">
-        <v>0.0316829561653608</v>
+        <v>0.0963577950755796</v>
       </c>
       <c r="G20" t="n">
-        <v>0.00107070820127441</v>
+        <v>-0.00239010461365922</v>
       </c>
       <c r="H20" t="n">
-        <v>0.0106235839530385</v>
+        <v>0.0194404087685528</v>
       </c>
       <c r="I20" t="n">
         <v>0.95</v>
       </c>
       <c r="J20" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="K20" t="n">
         <v>0</v>
@@ -1123,25 +1123,25 @@
         <v>0.000126484178421768</v>
       </c>
       <c r="D21" t="n">
-        <v>0.00368483649875352</v>
+        <v>0.0047514582395449</v>
       </c>
       <c r="E21" t="n">
-        <v>0.0343255877064164</v>
+        <v>0.0266200757841203</v>
       </c>
       <c r="F21" t="n">
-        <v>0.972617520850085</v>
+        <v>0.978762760772665</v>
       </c>
       <c r="G21" t="n">
-        <v>-0.00236132035285508</v>
+        <v>-0.00629287285558535</v>
       </c>
       <c r="H21" t="n">
-        <v>0.00653046176796185</v>
+        <v>0.0105163177670131</v>
       </c>
       <c r="I21" t="n">
         <v>0.95</v>
       </c>
       <c r="J21" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="K21" t="n">
         <v>0</v>
@@ -1158,25 +1158,25 @@
         <v>0.0223135358283244</v>
       </c>
       <c r="D22" t="n">
-        <v>0.00676891297143501</v>
+        <v>0.00553278379416509</v>
       </c>
       <c r="E22" t="n">
-        <v>3.29647255364165</v>
+        <v>4.03296724731165</v>
       </c>
       <c r="F22" t="n">
-        <v>0.000979071804916892</v>
+        <v>0.0000550769585354085</v>
       </c>
       <c r="G22" t="n">
-        <v>0.00813232299989102</v>
+        <v>0.00990342693350234</v>
       </c>
       <c r="H22" t="n">
-        <v>0.0250602925417596</v>
+        <v>0.032465560972016</v>
       </c>
       <c r="I22" t="n">
         <v>0.95</v>
       </c>
       <c r="J22" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="K22" t="n">
         <v>0</v>
@@ -1193,25 +1193,25 @@
         <v>-0.0490366814132291</v>
       </c>
       <c r="D23" t="n">
-        <v>0.00308558146925971</v>
+        <v>0.00490865538931612</v>
       </c>
       <c r="E23" t="n">
-        <v>-15.8922011626528</v>
+        <v>-9.98983988975055</v>
       </c>
       <c r="F23" t="n">
-        <v>0.00000000000000000000000000000000000000000000000000000000717627595980134</v>
+        <v>0.0000000000000000000000168854258879365</v>
       </c>
       <c r="G23" t="n">
-        <v>-0.0541271818539211</v>
+        <v>-0.059467229224725</v>
       </c>
       <c r="H23" t="n">
-        <v>-0.0474113989174505</v>
+        <v>-0.0425891103960169</v>
       </c>
       <c r="I23" t="n">
         <v>0.95</v>
       </c>
       <c r="J23" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="K23" t="n">
         <v>0</v>
@@ -1228,25 +1228,25 @@
         <v>-0.0628045477509041</v>
       </c>
       <c r="D24" t="n">
-        <v>0.0056776687199725</v>
+        <v>0.00547100489595562</v>
       </c>
       <c r="E24" t="n">
-        <v>-11.0616788066508</v>
+        <v>-11.4795268776549</v>
       </c>
       <c r="F24" t="n">
-        <v>0.000000000000000000000000000192461032720043</v>
+        <v>0.00000000000000000000000000000167192892702215</v>
       </c>
       <c r="G24" t="n">
-        <v>-0.0708008407407425</v>
+        <v>-0.0738841295229442</v>
       </c>
       <c r="H24" t="n">
-        <v>-0.0564464606296914</v>
+        <v>-0.0547004000563214</v>
       </c>
       <c r="I24" t="n">
         <v>0.95</v>
       </c>
       <c r="J24" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="K24" t="n">
         <v>0</v>
@@ -1263,25 +1263,25 @@
         <v>0.0428952462862584</v>
       </c>
       <c r="D25" t="n">
-        <v>0.00501830900354874</v>
+        <v>0.00463417834830771</v>
       </c>
       <c r="E25" t="n">
-        <v>8.54774910351767</v>
+        <v>9.25627868895522</v>
       </c>
       <c r="F25" t="n">
-        <v>0.0000000000000000125512188978144</v>
+        <v>0.0000000000000000000211681318765906</v>
       </c>
       <c r="G25" t="n">
-        <v>0.0321044075615251</v>
+        <v>0.0318106421618741</v>
       </c>
       <c r="H25" t="n">
-        <v>0.0442184094793397</v>
+        <v>0.0503166222064027</v>
       </c>
       <c r="I25" t="n">
         <v>0.95</v>
       </c>
       <c r="J25" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="K25" t="n">
         <v>0</v>
@@ -1298,25 +1298,25 @@
         <v>0.00846059229042843</v>
       </c>
       <c r="D26" t="n">
-        <v>0.00272989858044194</v>
+        <v>0.00325186313154537</v>
       </c>
       <c r="E26" t="n">
-        <v>3.09923319168097</v>
+        <v>2.60176764770777</v>
       </c>
       <c r="F26" t="n">
-        <v>0.00194022243343123</v>
+        <v>0.00927446644138081</v>
       </c>
       <c r="G26" t="n">
-        <v>0.00597776146390326</v>
+        <v>0.00385151795461758</v>
       </c>
       <c r="H26" t="n">
-        <v>0.012839625456855</v>
+        <v>0.0144515820428767</v>
       </c>
       <c r="I26" t="n">
         <v>0.95</v>
       </c>
       <c r="J26" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="K26" t="n">
         <v>0</v>
@@ -1333,25 +1333,25 @@
         <v>-0.00172636407818444</v>
       </c>
       <c r="D27" t="n">
-        <v>0.00137540063475581</v>
+        <v>0.00184711360807437</v>
       </c>
       <c r="E27" t="n">
-        <v>-1.25517179108395</v>
+        <v>-0.934627989657978</v>
       </c>
       <c r="F27" t="n">
-        <v>0.209416403494597</v>
+        <v>0.349980049284346</v>
       </c>
       <c r="G27" t="n">
-        <v>-0.00398236998914427</v>
+        <v>-0.00443830996472556</v>
       </c>
       <c r="H27" t="n">
-        <v>-0.000693787474654978</v>
+        <v>0.0027497981140109</v>
       </c>
       <c r="I27" t="n">
         <v>0.95</v>
       </c>
       <c r="J27" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="K27" t="n">
         <v>0</v>
@@ -1368,25 +1368,25 @@
         <v>0.0109257089390214</v>
       </c>
       <c r="D28" t="n">
-        <v>0.00166065236889214</v>
+        <v>0.00272443222664997</v>
       </c>
       <c r="E28" t="n">
-        <v>6.5791668043747</v>
+        <v>4.01027004164309</v>
       </c>
       <c r="F28" t="n">
-        <v>0.0000000000473091798780659</v>
+        <v>0.0000606493435612117</v>
       </c>
       <c r="G28" t="n">
-        <v>0.00876114544382582</v>
+        <v>0.00527251042920171</v>
       </c>
       <c r="H28" t="n">
-        <v>0.012884393899547</v>
+        <v>0.0160163465599095</v>
       </c>
       <c r="I28" t="n">
         <v>0.95</v>
       </c>
       <c r="J28" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="K28" t="n">
         <v>0</v>
@@ -1403,25 +1403,25 @@
         <v>-0.0239655762011174</v>
       </c>
       <c r="D29" t="n">
-        <v>0.00328335112295613</v>
+        <v>0.00361278509171776</v>
       </c>
       <c r="E29" t="n">
-        <v>-7.29912071650144</v>
+        <v>-6.6335460296429</v>
       </c>
       <c r="F29" t="n">
-        <v>0.00000000000028965435887219</v>
+        <v>0.0000000000327716714752991</v>
       </c>
       <c r="G29" t="n">
-        <v>-0.0250438455288243</v>
+        <v>-0.0312542188403483</v>
       </c>
       <c r="H29" t="n">
-        <v>-0.016827859097923</v>
+        <v>-0.016933485509261</v>
       </c>
       <c r="I29" t="n">
         <v>0.95</v>
       </c>
       <c r="J29" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="K29" t="n">
         <v>0</v>
@@ -1438,25 +1438,25 @@
         <v>-0.0286863684128684</v>
       </c>
       <c r="D30" t="n">
-        <v>0.00390663176724445</v>
+        <v>0.00412318832551333</v>
       </c>
       <c r="E30" t="n">
-        <v>-7.3429926652909</v>
+        <v>-6.95732674526746</v>
       </c>
       <c r="F30" t="n">
-        <v>0.000000000000208869978307238</v>
+        <v>0.00000000000346790021334142</v>
       </c>
       <c r="G30" t="n">
-        <v>-0.0324264296966277</v>
+        <v>-0.0373554905792666</v>
       </c>
       <c r="H30" t="n">
-        <v>-0.024643110242738</v>
+        <v>-0.0216440257530807</v>
       </c>
       <c r="I30" t="n">
         <v>0.95</v>
       </c>
       <c r="J30" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="K30" t="n">
         <v>0</v>
@@ -1473,25 +1473,25 @@
         <v>0.0173697388994499</v>
       </c>
       <c r="D31" t="n">
-        <v>0.00134811214907783</v>
+        <v>0.00255217842095071</v>
       </c>
       <c r="E31" t="n">
-        <v>12.8844910353576</v>
+        <v>6.80584819496262</v>
       </c>
       <c r="F31" t="n">
-        <v>0.0000000000000000000000000000000000000550373865297291</v>
+        <v>0.0000000000100455596931332</v>
       </c>
       <c r="G31" t="n">
-        <v>0.016463270871134</v>
+        <v>0.0125950170242982</v>
       </c>
       <c r="H31" t="n">
-        <v>0.0194253249513179</v>
+        <v>0.0230060034767627</v>
       </c>
       <c r="I31" t="n">
         <v>0.95</v>
       </c>
       <c r="J31" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="K31" t="n">
         <v>0</v>
@@ -1508,25 +1508,25 @@
         <v>0.00735974585595936</v>
       </c>
       <c r="D32" t="n">
-        <v>0.00769153049077956</v>
+        <v>0.00419085946509972</v>
       </c>
       <c r="E32" t="n">
-        <v>0.956863639139449</v>
+        <v>1.75614236584386</v>
       </c>
       <c r="F32" t="n">
-        <v>0.338636086001389</v>
+        <v>0.0790641027433782</v>
       </c>
       <c r="G32" t="n">
-        <v>-0.00383300921856239</v>
+        <v>-0.000950608507304957</v>
       </c>
       <c r="H32" t="n">
-        <v>0.0135410433520752</v>
+        <v>0.0145883098539944</v>
       </c>
       <c r="I32" t="n">
         <v>0.95</v>
       </c>
       <c r="J32" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="K32" t="n">
         <v>0</v>
@@ -1543,25 +1543,25 @@
         <v>-0.00097143002595742</v>
       </c>
       <c r="D33" t="n">
-        <v>0.00341722927058037</v>
+        <v>0.00370383204489166</v>
       </c>
       <c r="E33" t="n">
-        <v>-0.284274173325349</v>
+        <v>-0.262277018553587</v>
       </c>
       <c r="F33" t="n">
-        <v>0.77620027673996</v>
+        <v>0.793107878557127</v>
       </c>
       <c r="G33" t="n">
-        <v>-0.00480505587269475</v>
+        <v>-0.00849057686818316</v>
       </c>
       <c r="H33" t="n">
-        <v>0.00254337806731352</v>
+        <v>0.00460579776951946</v>
       </c>
       <c r="I33" t="n">
         <v>0.95</v>
       </c>
       <c r="J33" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="K33" t="n">
         <v>0</v>
@@ -1578,25 +1578,25 @@
         <v>0.0119254732947933</v>
       </c>
       <c r="D34" t="n">
-        <v>0.0044275276352057</v>
+        <v>0.0038956934118475</v>
       </c>
       <c r="E34" t="n">
-        <v>2.69348364987433</v>
+        <v>3.06119399912884</v>
       </c>
       <c r="F34" t="n">
-        <v>0.00707096134588109</v>
+        <v>0.00220456204418566</v>
       </c>
       <c r="G34" t="n">
-        <v>0.00931533855714362</v>
+        <v>0.00618741299292924</v>
       </c>
       <c r="H34" t="n">
-        <v>0.0193924518590467</v>
+        <v>0.0196187030784897</v>
       </c>
       <c r="I34" t="n">
         <v>0.95</v>
       </c>
       <c r="J34" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="K34" t="n">
         <v>0</v>
@@ -1613,25 +1613,25 @@
         <v>-0.0351705897822556</v>
       </c>
       <c r="D35" t="n">
-        <v>0.00345931286763776</v>
+        <v>0.00495603600244948</v>
       </c>
       <c r="E35" t="n">
-        <v>-10.1669294244184</v>
+        <v>-7.09651620062341</v>
       </c>
       <c r="F35" t="n">
-        <v>0.00000000000000000000000278551530510328</v>
+        <v>0.00000000000127940955558876</v>
       </c>
       <c r="G35" t="n">
-        <v>-0.040445707463237</v>
+        <v>-0.0436289204580704</v>
       </c>
       <c r="H35" t="n">
-        <v>-0.0327038712352013</v>
+        <v>-0.0258277871013219</v>
       </c>
       <c r="I35" t="n">
         <v>0.95</v>
       </c>
       <c r="J35" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="K35" t="n">
         <v>0</v>
@@ -1648,25 +1648,25 @@
         <v>-0.0431291031359325</v>
       </c>
       <c r="D36" t="n">
-        <v>0.00293855731118729</v>
+        <v>0.00518144991999209</v>
       </c>
       <c r="E36" t="n">
-        <v>-14.6769651120082</v>
+        <v>-8.32375180729303</v>
       </c>
       <c r="F36" t="n">
-        <v>0.000000000000000000000000000000000000000000000000905536076040891</v>
+        <v>0.0000000000000000852219543995958</v>
       </c>
       <c r="G36" t="n">
-        <v>-0.0438973506700162</v>
+        <v>-0.0503540053025753</v>
       </c>
       <c r="H36" t="n">
-        <v>-0.0377198750508405</v>
+        <v>-0.0312236070622654</v>
       </c>
       <c r="I36" t="n">
         <v>0.95</v>
       </c>
       <c r="J36" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="K36" t="n">
         <v>0</v>
@@ -1683,25 +1683,25 @@
         <v>0.0340466100667462</v>
       </c>
       <c r="D37" t="n">
-        <v>0.00474720150787267</v>
+        <v>0.00366688340401564</v>
       </c>
       <c r="E37" t="n">
-        <v>7.17193277139889</v>
+        <v>9.28489027752053</v>
       </c>
       <c r="F37" t="n">
-        <v>0.000000000000739462558128237</v>
+        <v>0.0000000000000000000161873872878594</v>
       </c>
       <c r="G37" t="n">
-        <v>0.0279073376523744</v>
+        <v>0.0274782137370368</v>
       </c>
       <c r="H37" t="n">
-        <v>0.0397458058667633</v>
+        <v>0.0402978229346208</v>
       </c>
       <c r="I37" t="n">
         <v>0.95</v>
       </c>
       <c r="J37" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="K37" t="n">
         <v>0</v>
@@ -1718,25 +1718,25 @@
         <v>0.0161507573011293</v>
       </c>
       <c r="D38" t="n">
-        <v>0.00794542244649332</v>
+        <v>0.00565813040555709</v>
       </c>
       <c r="E38" t="n">
-        <v>2.03271222013593</v>
+        <v>2.85443355728723</v>
       </c>
       <c r="F38" t="n">
-        <v>0.0420816059642567</v>
+        <v>0.00431136489943116</v>
       </c>
       <c r="G38" t="n">
-        <v>0.00937535695751416</v>
+        <v>0.0061687110125481</v>
       </c>
       <c r="H38" t="n">
-        <v>0.0279602574878762</v>
+        <v>0.0279686186749325</v>
       </c>
       <c r="I38" t="n">
         <v>0.95</v>
       </c>
       <c r="J38" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="K38" t="n">
         <v>0</v>
@@ -1753,25 +1753,25 @@
         <v>-0.00212544779163588</v>
       </c>
       <c r="D39" t="n">
-        <v>0.00627327836476059</v>
+        <v>0.00503790066062404</v>
       </c>
       <c r="E39" t="n">
-        <v>-0.338809736799715</v>
+        <v>-0.42189156452573</v>
       </c>
       <c r="F39" t="n">
-        <v>0.734753065768298</v>
+        <v>0.673104167451147</v>
       </c>
       <c r="G39" t="n">
-        <v>-0.00633868237204883</v>
+        <v>-0.00944598163666887</v>
       </c>
       <c r="H39" t="n">
-        <v>0.00817180246324503</v>
+        <v>0.00902983550645525</v>
       </c>
       <c r="I39" t="n">
         <v>0.95</v>
       </c>
       <c r="J39" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="K39" t="n">
         <v>0</v>
@@ -1788,25 +1788,25 @@
         <v>0.0221833428986292</v>
       </c>
       <c r="D40" t="n">
-        <v>0.00344601295175515</v>
+        <v>0.00580425219852934</v>
       </c>
       <c r="E40" t="n">
-        <v>6.43739394169444</v>
+        <v>3.82191230495634</v>
       </c>
       <c r="F40" t="n">
-        <v>0.000000000121542191845516</v>
+        <v>0.000132420784234566</v>
       </c>
       <c r="G40" t="n">
-        <v>0.0187194635532134</v>
+        <v>0.0105387806469837</v>
       </c>
       <c r="H40" t="n">
-        <v>0.0262065452977974</v>
+        <v>0.0307174102964294</v>
       </c>
       <c r="I40" t="n">
         <v>0.95</v>
       </c>
       <c r="J40" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="K40" t="n">
         <v>0</v>
@@ -1823,25 +1823,25 @@
         <v>-0.0585962123638953</v>
       </c>
       <c r="D41" t="n">
-        <v>0.00611451523960419</v>
+        <v>0.00725349207115189</v>
       </c>
       <c r="E41" t="n">
-        <v>-9.58313293331303</v>
+        <v>-8.07834513212475</v>
       </c>
       <c r="F41" t="n">
-        <v>0.000000000000000000000941449403761789</v>
+        <v>0.00000000000000065651579808417</v>
       </c>
       <c r="G41" t="n">
-        <v>-0.0634861661387777</v>
+        <v>-0.0712584348066616</v>
       </c>
       <c r="H41" t="n">
-        <v>-0.0497740293608378</v>
+        <v>-0.0486957253591848</v>
       </c>
       <c r="I41" t="n">
         <v>0.95</v>
       </c>
       <c r="J41" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="K41" t="n">
         <v>0</v>
@@ -1858,25 +1858,25 @@
         <v>-0.0728927684731198</v>
       </c>
       <c r="D42" t="n">
-        <v>0.00661396481618285</v>
+        <v>0.00823320263945239</v>
       </c>
       <c r="E42" t="n">
-        <v>-11.0210396485279</v>
+        <v>-8.85351322750487</v>
       </c>
       <c r="F42" t="n">
-        <v>0.000000000000000000000000000302544337840234</v>
+        <v>0.000000000000000000848066282180469</v>
       </c>
       <c r="G42" t="n">
-        <v>-0.0765289726597496</v>
+        <v>-0.0860068867528369</v>
       </c>
       <c r="H42" t="n">
-        <v>-0.0600639985849651</v>
+        <v>-0.0578436873532468</v>
       </c>
       <c r="I42" t="n">
         <v>0.95</v>
       </c>
       <c r="J42" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="K42" t="n">
         <v>0</v>
@@ -1893,25 +1893,25 @@
         <v>0.0509752066652773</v>
       </c>
       <c r="D43" t="n">
-        <v>0.00470463967274518</v>
+        <v>0.00449043850059483</v>
       </c>
       <c r="E43" t="n">
-        <v>10.8350926343171</v>
+        <v>11.3519440603685</v>
       </c>
       <c r="F43" t="n">
-        <v>0.00000000000000000000000000234727722924487</v>
+        <v>0.00000000000000000000000000000725318416634008</v>
       </c>
       <c r="G43" t="n">
-        <v>0.0474116028000342</v>
+        <v>0.0440009875103712</v>
       </c>
       <c r="H43" t="n">
-        <v>0.0575598262797791</v>
+        <v>0.0598452193209655</v>
       </c>
       <c r="I43" t="n">
         <v>0.95</v>
       </c>
       <c r="J43" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="K43" t="n">
         <v>0</v>

</xml_diff>